<commit_message>
Agrega resultados de simulación y actualizaciones de código
</commit_message>
<xml_diff>
--- a/scripts/simulations/resultados_simulacion/Grupo3_Mezclas/mse_puntual_mezcla_mw_n120.xlsx
+++ b/scripts/simulations/resultados_simulacion/Grupo3_Mezclas/mse_puntual_mezcla_mw_n120.xlsx
@@ -410,20 +410,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Moda</t>
+          <t>P05</t>
         </is>
       </c>
       <c r="E2">
-        <v>0.00211542945234218</v>
+        <v>0.0004041293866167073</v>
       </c>
       <c r="F2">
-        <v>0.001573913294337817</v>
+        <v>0.000636414287854239</v>
       </c>
       <c r="G2">
-        <v>0.001326857711787192</v>
+        <v>0.0005723373717965813</v>
       </c>
       <c r="H2">
-        <v>0.003160306023542861</v>
+        <v>0.0003392926218097917</v>
       </c>
     </row>
     <row r="3">
@@ -440,20 +440,20 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>Moda_Izq</t>
         </is>
       </c>
       <c r="E3">
-        <v>0.0004041293866167073</v>
+        <v>0.002052045280909065</v>
       </c>
       <c r="F3">
-        <v>0.000636414287854239</v>
+        <v>0.001631937114555233</v>
       </c>
       <c r="G3">
-        <v>0.0005723373717965813</v>
+        <v>0.001303743158338</v>
       </c>
       <c r="H3">
-        <v>0.0003392926218097917</v>
+        <v>0.003119258413875391</v>
       </c>
     </row>
     <row r="4">
@@ -470,20 +470,20 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Valle_Central</t>
         </is>
       </c>
       <c r="E4">
-        <v>0.002052064881447446</v>
+        <v>0.001382714841782616</v>
       </c>
       <c r="F4">
-        <v>0.001631981443390887</v>
+        <v>0.0006591235295379591</v>
       </c>
       <c r="G4">
-        <v>0.001303762556129341</v>
+        <v>0.0006096160080590804</v>
       </c>
       <c r="H4">
-        <v>0.003119273583667888</v>
+        <v>0.002395311163443158</v>
       </c>
     </row>
     <row r="5">
@@ -500,20 +500,20 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Mediana</t>
+          <t>Moda_Der</t>
         </is>
       </c>
       <c r="E5">
-        <v>0.001382714841782614</v>
+        <v>0.00211542945234218</v>
       </c>
       <c r="F5">
-        <v>0.0006591235295379587</v>
+        <v>0.001573913294337817</v>
       </c>
       <c r="G5">
-        <v>0.0006096160080590801</v>
+        <v>0.001326857711787192</v>
       </c>
       <c r="H5">
-        <v>0.002395311163443156</v>
+        <v>0.003160306023542861</v>
       </c>
     </row>
     <row r="6">
@@ -590,20 +590,20 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Moda</t>
+          <t>Garra_1</t>
         </is>
       </c>
       <c r="E8">
-        <v>0.04466923766304482</v>
+        <v>0.0581545622393735</v>
       </c>
       <c r="F8">
-        <v>0.02942786499929357</v>
+        <v>0.03136951460517007</v>
       </c>
       <c r="G8">
-        <v>0.04560817097794589</v>
+        <v>0.05697414014611751</v>
       </c>
       <c r="H8">
-        <v>0.06252492160782844</v>
+        <v>0.06892027957289441</v>
       </c>
     </row>
     <row r="9">
@@ -620,20 +620,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>Garra_2</t>
         </is>
       </c>
       <c r="E9">
-        <v>0.008810450827054585</v>
+        <v>0.04477834278469823</v>
       </c>
       <c r="F9">
-        <v>0.005022296877974886</v>
+        <v>0.02952750415509241</v>
       </c>
       <c r="G9">
-        <v>0.008640355679978588</v>
+        <v>0.04537895858657231</v>
       </c>
       <c r="H9">
-        <v>0.009272476267128966</v>
+        <v>0.06691503534339791</v>
       </c>
     </row>
     <row r="10">
@@ -650,20 +650,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Garra_3</t>
         </is>
       </c>
       <c r="E10">
-        <v>0.003273096265065665</v>
+        <v>0.04466923766304483</v>
       </c>
       <c r="F10">
-        <v>0.009600262885137278</v>
+        <v>0.02942786499929317</v>
       </c>
       <c r="G10">
-        <v>0.003689290722606258</v>
+        <v>0.04560817097794596</v>
       </c>
       <c r="H10">
-        <v>0.01202621506432443</v>
+        <v>0.06252492160782856</v>
       </c>
     </row>
     <row r="11">
@@ -680,20 +680,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Mediana</t>
+          <t>Garra_4</t>
         </is>
       </c>
       <c r="E11">
-        <v>0.04466923766304483</v>
+        <v>0.04392135353739618</v>
       </c>
       <c r="F11">
-        <v>0.02942786499929317</v>
+        <v>0.02936934553309585</v>
       </c>
       <c r="G11">
-        <v>0.04560817097794596</v>
+        <v>0.04465285607647237</v>
       </c>
       <c r="H11">
-        <v>0.06252492160782856</v>
+        <v>0.06521917481888015</v>
       </c>
     </row>
     <row r="12">
@@ -710,20 +710,20 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Garra_5</t>
         </is>
       </c>
       <c r="E12">
-        <v>0.003239387831356956</v>
+        <v>0.05764844717471663</v>
       </c>
       <c r="F12">
-        <v>0.009540547598969964</v>
+        <v>0.03086051382572902</v>
       </c>
       <c r="G12">
-        <v>0.003624449036549287</v>
+        <v>0.05645569825908689</v>
       </c>
       <c r="H12">
-        <v>0.01172575866115142</v>
+        <v>0.06758068392930792</v>
       </c>
     </row>
     <row r="13">
@@ -770,20 +770,20 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Moda</t>
+          <t>P05</t>
         </is>
       </c>
       <c r="E14">
-        <v>0.002128873001368338</v>
+        <v>0.0004956832843639399</v>
       </c>
       <c r="F14">
-        <v>0.001649356488399976</v>
+        <v>0.000749556621822574</v>
       </c>
       <c r="G14">
-        <v>0.001435305074710627</v>
+        <v>0.0006761051085019963</v>
       </c>
       <c r="H14">
-        <v>0.003415507908042497</v>
+        <v>0.0003794837593292449</v>
       </c>
     </row>
     <row r="15">
@@ -800,20 +800,20 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>Moda_Izq</t>
         </is>
       </c>
       <c r="E15">
-        <v>0.0004956832843639399</v>
+        <v>0.00223025653523031</v>
       </c>
       <c r="F15">
-        <v>0.000749556621822574</v>
+        <v>0.001704509324838449</v>
       </c>
       <c r="G15">
-        <v>0.0006761051085019963</v>
+        <v>0.001482047667080107</v>
       </c>
       <c r="H15">
-        <v>0.0003794837593292449</v>
+        <v>0.003542439095532733</v>
       </c>
     </row>
     <row r="16">
@@ -830,20 +830,20 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Valle_Central</t>
         </is>
       </c>
       <c r="E16">
-        <v>0.002230287682613931</v>
+        <v>0.001394737545519829</v>
       </c>
       <c r="F16">
-        <v>0.001704558830477491</v>
+        <v>0.0006820991007851654</v>
       </c>
       <c r="G16">
-        <v>0.001482074518341558</v>
+        <v>0.0006277896651409987</v>
       </c>
       <c r="H16">
-        <v>0.003542494060984201</v>
+        <v>0.002601346622947196</v>
       </c>
     </row>
     <row r="17">
@@ -860,20 +860,20 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Mediana</t>
+          <t>Moda_Der</t>
         </is>
       </c>
       <c r="E17">
-        <v>0.001394737545519828</v>
+        <v>0.002128873001368338</v>
       </c>
       <c r="F17">
-        <v>0.0006820991007851647</v>
+        <v>0.001649356488399976</v>
       </c>
       <c r="G17">
-        <v>0.0006277896651409982</v>
+        <v>0.001435305074710627</v>
       </c>
       <c r="H17">
-        <v>0.002601346622947195</v>
+        <v>0.003415507908042497</v>
       </c>
     </row>
     <row r="18">
@@ -950,20 +950,20 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Moda</t>
+          <t>Garra_1</t>
         </is>
       </c>
       <c r="E20">
-        <v>0.0451345824124845</v>
+        <v>0.05835143891465377</v>
       </c>
       <c r="F20">
-        <v>0.03098002284993808</v>
+        <v>0.03310715910489749</v>
       </c>
       <c r="G20">
-        <v>0.04596361374160898</v>
+        <v>0.05713943391433156</v>
       </c>
       <c r="H20">
-        <v>0.08640314872515917</v>
+        <v>0.08326472706680808</v>
       </c>
     </row>
     <row r="21">
@@ -980,20 +980,20 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>Garra_2</t>
         </is>
       </c>
       <c r="E21">
-        <v>0.009531701693203441</v>
+        <v>0.04408066311122617</v>
       </c>
       <c r="F21">
-        <v>0.005377029806031936</v>
+        <v>0.02869653724697161</v>
       </c>
       <c r="G21">
-        <v>0.009298420337562518</v>
+        <v>0.04444419220183153</v>
       </c>
       <c r="H21">
-        <v>0.009569198101070171</v>
+        <v>0.08495230579594687</v>
       </c>
     </row>
     <row r="22">
@@ -1010,20 +1010,20 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Garra_3</t>
         </is>
       </c>
       <c r="E22">
-        <v>0.003812569431432427</v>
+        <v>0.0451345824124845</v>
       </c>
       <c r="F22">
-        <v>0.01062999035905333</v>
+        <v>0.03098002284993804</v>
       </c>
       <c r="G22">
-        <v>0.004080369047662065</v>
+        <v>0.04596361374160893</v>
       </c>
       <c r="H22">
-        <v>0.01433479495917032</v>
+        <v>0.08640314872515918</v>
       </c>
     </row>
     <row r="23">
@@ -1040,20 +1040,20 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Mediana</t>
+          <t>Garra_4</t>
         </is>
       </c>
       <c r="E23">
-        <v>0.0451345824124845</v>
+        <v>0.04522153924078236</v>
       </c>
       <c r="F23">
-        <v>0.03098002284993804</v>
+        <v>0.02899886407705054</v>
       </c>
       <c r="G23">
-        <v>0.04596361374160893</v>
+        <v>0.04607515625014758</v>
       </c>
       <c r="H23">
-        <v>0.08640314872515918</v>
+        <v>0.08532154559250316</v>
       </c>
     </row>
     <row r="24">
@@ -1070,20 +1070,20 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Garra_5</t>
         </is>
       </c>
       <c r="E24">
-        <v>0.003960128108878542</v>
+        <v>0.05937471374615225</v>
       </c>
       <c r="F24">
-        <v>0.01031073082360688</v>
+        <v>0.03327993722113175</v>
       </c>
       <c r="G24">
-        <v>0.004258468605436381</v>
+        <v>0.05778805663365198</v>
       </c>
       <c r="H24">
-        <v>0.01452079599828362</v>
+        <v>0.08415619534858261</v>
       </c>
     </row>
     <row r="25">
@@ -1130,20 +1130,20 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Moda</t>
+          <t>P05</t>
         </is>
       </c>
       <c r="E26">
-        <v>0.004840846047501489</v>
+        <v>0.003100900704075873</v>
       </c>
       <c r="F26">
-        <v>0.005451503233107791</v>
+        <v>0.004423303419501327</v>
       </c>
       <c r="G26">
-        <v>0.005022208665680052</v>
+        <v>0.004091430546216258</v>
       </c>
       <c r="H26">
-        <v>0.005798996805424811</v>
+        <v>0.002290652543107791</v>
       </c>
     </row>
     <row r="27">
@@ -1160,20 +1160,20 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>Moda_Izq</t>
         </is>
       </c>
       <c r="E27">
-        <v>0.003100900704075873</v>
+        <v>0.004445470281331766</v>
       </c>
       <c r="F27">
-        <v>0.004423303419501327</v>
+        <v>0.005114375462145964</v>
       </c>
       <c r="G27">
-        <v>0.004091430546216258</v>
+        <v>0.004697224164210659</v>
       </c>
       <c r="H27">
-        <v>0.002290652543107791</v>
+        <v>0.005307868803520271</v>
       </c>
     </row>
     <row r="28">
@@ -1190,20 +1190,20 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Valle_Central</t>
         </is>
       </c>
       <c r="E28">
-        <v>0.004445628667270193</v>
+        <v>0.001542115406324752</v>
       </c>
       <c r="F28">
-        <v>0.005114663807625591</v>
+        <v>0.0009585214007194658</v>
       </c>
       <c r="G28">
-        <v>0.004697434965514107</v>
+        <v>0.0008810685125765294</v>
       </c>
       <c r="H28">
-        <v>0.005300605014419043</v>
+        <v>0.0031484914680002</v>
       </c>
     </row>
     <row r="29">
@@ -1220,20 +1220,20 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Mediana</t>
+          <t>Moda_Der</t>
         </is>
       </c>
       <c r="E29">
-        <v>0.001542115406324752</v>
+        <v>0.004840846047501489</v>
       </c>
       <c r="F29">
-        <v>0.0009585214007194651</v>
+        <v>0.005451503233107791</v>
       </c>
       <c r="G29">
-        <v>0.0008810685125765289</v>
+        <v>0.005022208665680052</v>
       </c>
       <c r="H29">
-        <v>0.003148491468000199</v>
+        <v>0.005798996805424811</v>
       </c>
     </row>
     <row r="30">
@@ -1310,20 +1310,20 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Moda</t>
+          <t>Garra_1</t>
         </is>
       </c>
       <c r="E32">
-        <v>0.05289022634720938</v>
+        <v>0.07479532972500383</v>
       </c>
       <c r="F32">
-        <v>0.04758525990003452</v>
+        <v>0.07155019078990077</v>
       </c>
       <c r="G32">
-        <v>0.053845588925822</v>
+        <v>0.07615912627937901</v>
       </c>
       <c r="H32">
-        <v>0.08153792693321939</v>
+        <v>0.08298315619801712</v>
       </c>
     </row>
     <row r="33">
@@ -1340,20 +1340,20 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>Garra_2</t>
         </is>
       </c>
       <c r="E33">
-        <v>0.01643580755894435</v>
+        <v>0.05470745460145469</v>
       </c>
       <c r="F33">
-        <v>0.01076714751630739</v>
+        <v>0.04824080501286957</v>
       </c>
       <c r="G33">
-        <v>0.01507446609719142</v>
+        <v>0.05500760259956515</v>
       </c>
       <c r="H33">
-        <v>0.01112289007248105</v>
+        <v>0.08101832453294101</v>
       </c>
     </row>
     <row r="34">
@@ -1370,20 +1370,20 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Garra_3</t>
         </is>
       </c>
       <c r="E34">
-        <v>0.01505850179970785</v>
+        <v>0.05289022634720941</v>
       </c>
       <c r="F34">
-        <v>0.02458985975399679</v>
+        <v>0.04758525990003386</v>
       </c>
       <c r="G34">
-        <v>0.0164236552333524</v>
+        <v>0.05384558892582204</v>
       </c>
       <c r="H34">
-        <v>0.0159062645287428</v>
+        <v>0.08153792693321944</v>
       </c>
     </row>
     <row r="35">
@@ -1400,20 +1400,20 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Mediana</t>
+          <t>Garra_4</t>
         </is>
       </c>
       <c r="E35">
-        <v>0.05289022634720941</v>
+        <v>0.05295730042796341</v>
       </c>
       <c r="F35">
-        <v>0.04758525990003386</v>
+        <v>0.04776087698231792</v>
       </c>
       <c r="G35">
-        <v>0.05384558892582204</v>
+        <v>0.05408136474637814</v>
       </c>
       <c r="H35">
-        <v>0.08153792693321944</v>
+        <v>0.08021116626899648</v>
       </c>
     </row>
     <row r="36">
@@ -1430,20 +1430,20 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Garra_5</t>
         </is>
       </c>
       <c r="E36">
-        <v>0.01459259955892309</v>
+        <v>0.07073636176677851</v>
       </c>
       <c r="F36">
-        <v>0.0255475152442124</v>
+        <v>0.07167349985405207</v>
       </c>
       <c r="G36">
-        <v>0.01666835655924309</v>
+        <v>0.0732456679400799</v>
       </c>
       <c r="H36">
-        <v>0.01507559883147356</v>
+        <v>0.08020523613005949</v>
       </c>
     </row>
     <row r="37">

</xml_diff>